<commit_message>
Fix answer scripts to match exercise md requirements
step2_answer.py: rewrite to reflect CLAUDE.md harness rules (파일명 양식,
경비총괄표 시트, 일반/특별경비 분류, 접대비 비고 규칙, 개인카드 정산상태)
step3_answer.py: add 월별피벗 sheet for corp×month pivot table

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/week04-hands-on/data/법인매출통합.xlsx
+++ b/week04-hands-on/data/법인매출통합.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합데이터" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="법인별합계" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="월별피벗" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1003,4 +1004,140 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>법인명</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>독일</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>98000</v>
+      </c>
+      <c r="C2" t="n">
+        <v>105000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>101000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>304000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>125000</v>
+      </c>
+      <c r="C3" t="n">
+        <v>132000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>118000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>375000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>베트남</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3250000000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3480000000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3120000000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9850000000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>15800000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>16200000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>14900000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>46900000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>890000</v>
+      </c>
+      <c r="C6" t="n">
+        <v>920000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>875000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2685000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>